<commit_message>
refactor: refine schedule assistant, GA operators, benchmark suite and UI
</commit_message>
<xml_diff>
--- a/outputs/production/best_timetable.xlsx
+++ b/outputs/production/best_timetable.xlsx
@@ -688,7 +688,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>6.298559521092102</t>
+          <t>6.364253788022324</t>
         </is>
       </c>
     </row>
@@ -700,7 +700,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>6.298559521092102</t>
+          <t>6.364253788022324</t>
         </is>
       </c>
     </row>
@@ -928,7 +928,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 09:13:17</t>
+          <t>2026-08-12 07:01:34</t>
         </is>
       </c>
     </row>
@@ -24696,10 +24696,10 @@
         <v>1671</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>6.2986</v>
+        <v>6.3643</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>0.7369</v>
+        <v>0.7406</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>1000</v>

</xml_diff>